<commit_message>
Update: D19–D21 (name match, military enclaves, coastal strip)
</commit_message>
<xml_diff>
--- a/code/publicness_kurallar.xlsx
+++ b/code/publicness_kurallar.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="foursquare_sozluk" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="poi_temizlik" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kontrol" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="d19_adaylar" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="duzeltmeler" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'osm_kurallari'!$A$1:$G$136</definedName>
@@ -27,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,8 +109,11 @@
     <font>
       <color rgb="001A1A18"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="30">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -255,6 +260,11 @@
         <fgColor rgb="000F6E56"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF4CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -268,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -388,6 +398,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -755,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -912,6 +927,95 @@
       <c r="A25" t="inlineStr">
         <is>
           <t>zemin dışı: köprü, su, yol kaydı gibi mekân olmayan kayıtlar; hesaptan çıkar</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d19_adaylar: D19'un eşleştirdiği alanlar. KARAR boşsa önerilen rejim uygulanır; başka bir rejim yazılırsa o, 'uygulama' yazılırsa alan eskisi gibi kalır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>duzeltmeler: kuralların yakalayamadığı yerler. OSM no (w123 / r456) ya da OSM adı ve gerçek rejim; kaynak ve tarih yazılmalı. Düzeltme her şeyin (su hariç) üstüne boyanır.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>OSM no ya da ad</t>
+        </is>
+      </c>
+      <c r="B1" s="47" t="inlineStr">
+        <is>
+          <t>Rejim</t>
+        </is>
+      </c>
+      <c r="C1" s="47" t="inlineStr">
+        <is>
+          <t>Kaynak</t>
+        </is>
+      </c>
+      <c r="D1" s="47" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="E1" s="47" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Çubuklu Siloları</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>İBB kültür ve sergi mekânı; OSM'de eski petrol tankı etiketli</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bütün yerleşke, tank binaları dahil (müze kaydı tek tankı biletli yapıyordu)</t>
         </is>
       </c>
     </row>
@@ -926,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1716,6 +1820,132 @@
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Ad eşleşmesi alana rejim verir</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>uygula; uygulama</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>uygula</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Kuralı olmayan adlı bir OSM alanı (500 m²–100 ha), içinde ya da 25 m yakınında aynı adı taşıyan (benzerlik ≥0,85) temizlenmiş POI'lerin rejimini alır; en sık rejim, eşitlikte daha kamusal. Kafe, ATM, büfe gibi alt birimler sayılmaz. Kuralı olan alanlara dokunmaz. 51 aday: d19_adaylar sayfası. Çubuklu Siloları örneği.</t>
+        </is>
+      </c>
+      <c r="F20" s="40" t="inlineStr">
+        <is>
+          <t>karar verildi</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>uygula</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Askeri alan içindeki kamusal adalar</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>uygula; uygulama</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>uygula</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>OSM askeri sınırları kaba çiziliyor. Askeri poligon içinde ayrıca çizilmiş park, cami/cemevi, mezarlık, meydan (açık-kamusal alan ve binalar) askeri alandan önce boyanır. Hz. Yuşa Tepesi (Boğaz Komutanlığı poligonu içinde).</t>
+        </is>
+      </c>
+      <c r="F21" s="40" t="inlineStr">
+        <is>
+          <t>karar verildi</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>uygula</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Kıyı şeridi</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>30 m; 50 m; uygulama — Boğaz dahil/hariç</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>30 m, Boğaz hariç</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>3621 sayılı Kıyı Kanunu: kıyı herkesin eşit ve serbest yararlanmasına açık. Kıyıdan ilk 30 m'de OSM'nin boş bıraktığı zemin açık-kamusal sayılır (ayrı sınıf 'kıyı', modellendiği haritada görünür). Ölçüm: ilk 30 m'nin %47,5'i haritasızdı. Boğaz (Sarayburnu–Harem hattının kuzeyi) yalı bahçeleri riski yüzünden hariç.</t>
+        </is>
+      </c>
+      <c r="F22" s="40" t="inlineStr">
+        <is>
+          <t>karar verildi</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>30 m, Boğaz hariç</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
@@ -62941,4 +63171,1831 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
+      <c r="B1" s="47" t="inlineStr">
+        <is>
+          <t>OSM no</t>
+        </is>
+      </c>
+      <c r="C1" s="47" t="inlineStr">
+        <is>
+          <t>Alan (ha)</t>
+        </is>
+      </c>
+      <c r="D1" s="47" t="inlineStr">
+        <is>
+          <t>OSM etiketi</t>
+        </is>
+      </c>
+      <c r="E1" s="47" t="inlineStr">
+        <is>
+          <t>Önerilen rejim</t>
+        </is>
+      </c>
+      <c r="F1" s="47" t="inlineStr">
+        <is>
+          <t>Eşleşen kayıtlar</t>
+        </is>
+      </c>
+      <c r="G1" s="47" t="inlineStr">
+        <is>
+          <t>Dikkat</t>
+        </is>
+      </c>
+      <c r="H1" s="48" t="inlineStr">
+        <is>
+          <t>KARAR (siz)</t>
+        </is>
+      </c>
+      <c r="I1" s="48" t="inlineStr">
+        <is>
+          <t>NOT (siz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Maltepe Ceza İnfaz Kurumları Kampüsü</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>w281044271</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>41.94</v>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>amenity=prison</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Maltepe Ceza İnfaz Kurumları Kampüsü (foursquare, Prison, 1.0)</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="49" t="n"/>
+      <c r="I2" s="4" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Marintürk İstanbul City Port</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>w242415638</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>20.66</v>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>MarinTurk İstanbul City Port (foursquare, Harbor or Marina, 1.0)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H3" s="49" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>İETT İkitelli Garajı</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>w511777435</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>17.17</v>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>landuse=garages</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>I.E.T.T Ikitelli Garaji (foursquare, Bus Station, 0.93)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="49" t="n"/>
+      <c r="I4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Türkiye Futbol Federasyonu</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>w1429561728</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>landuse=sports</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Türkiye Futbol Federasyonu (overture, stadium_arena, 1.0)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="49" t="n"/>
+      <c r="I5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Metro İstanbul Behiç Erkin Yerleşkesi</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>w509910078</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>16.37</v>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>landuse=railway</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Metro İstanbul Behiç Erkin Yerleşkesi (foursquare, Metro Station, 1.0)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="49" t="n"/>
+      <c r="I6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Setur Fenerbahçe Marina</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>w236778445</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>15.26</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Fenerbahçe Marina (overture, marina, 0.85)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H7" s="49" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Setur Kalamış Marina</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>w242312415</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Setur Kalamış Marina A3 (foursquare, Harbor or Marina, 0.93) | Setur Kalamış Marina C2 (foursquare, Harbor or Marina, 0.93)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H8" s="49" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Demokrasi ve Özgürlük Adası</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>w144009911</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Demokrasi ve Özgürlükler Adası (overture, museum, 0.95)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Müze → biletli kuralından; adaya ulaşım ve giriş koşuluna göre.</t>
+        </is>
+      </c>
+      <c r="H9" s="49" t="n"/>
+      <c r="I9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Ümraniye Kapalı Cezaevi</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>w305843635</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>amenity=prison</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Ümraniye Kapalı Ceza Evi (overture, jail_or_prison, 0.98) | ümraniye T tipi kapalı cezaevi (foursquare, Prison, 0.87)</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="49" t="n"/>
+      <c r="I10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Ataköy Marina</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>w242413873</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>atakoy marina E39 (foursquare, Harbor or Marina, 0.87) | ATAKÖY MARİNA (foursquare, Harbor or Marina, 1.0)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H11" s="49" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Ataşehir Golf Club</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>w854955517</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>9.869999999999999</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>leisure=golf_course</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Atasehir Golf Club (overture, golf_course, 1.0)</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="49" t="n"/>
+      <c r="I12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Galataport</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>w343046405</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>landuse=harbour</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Galataport (foursquare, Harbor or Marina, 1.0)</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Sözlük 'Harbor or Marina'yı erişimsiz sayıyor; Galataport büyük ölçüde açık sahil aksı, özel işletme → yarı-kamusal olabilir.</t>
+        </is>
+      </c>
+      <c r="H13" s="49" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Metris Cezaevi</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>w499882134</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>amenity=prison</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Metris Cezaevi (foursquare, Prison, 1.0)</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="49" t="n"/>
+      <c r="I14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>İstinye Marina</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>w307333614</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>İstinye Marina (overture, marina, 1.0) | İstinye Marina (foursquare, Harbor or Marina, 1.0)</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H15" s="49" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Kanuni Sultan Süleyman Parkı</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>r8309769</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Kanuni Sultan Süleyman Parkı (foursquare, Park, 1.0)</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="49" t="n"/>
+      <c r="I16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Maltepe Huzurevi</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>w177449095</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>amenity=social_facility</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Maltepe Huzurevi (overture, senior_living_facility, 1.0) | Maltepe Huzurevi (foursquare, Non-Profit Organization, 1.0)</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="49" t="n"/>
+      <c r="I17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul Bilgi University</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>r0</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul Bilgi Üniversitesi (overture, college_university, 0.92)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="49" t="n"/>
+      <c r="I18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Tarabya Marina</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>w307333538</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Tarabya Marina (overture, marina, 1.0) | Tarabya Marina (foursquare, Harbor or Marina, 1.0)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H19" s="49" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>İETT Hasanpaşa Garajı</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>w202569515</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>landuse=garages</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>İETT Hasanpaşa Garajı (foursquare, Parking, 1.0)</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="49" t="n"/>
+      <c r="I20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Pera Kamping</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>r20353956</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>tourism=caravan_site</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Pera Camping (overture, rv_park, 0.92)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="49" t="n"/>
+      <c r="I21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Maltepe Karavan Park</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>w1506639021</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>tourism=caravan_site</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>yarı-kamusal</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Maltepe Karavan Park (foursquare, Campground, 1.0)</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="49" t="n"/>
+      <c r="I22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul Yelken Kulübü</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>w236167024</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>landuse=recreation_ground</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>istanbul yelken kulübü  Atölye (foursquare, Club House, 0.86) | İstanbul Yelken Kulübü (foursquare, Social Club, 1.0)</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="49" t="n"/>
+      <c r="I23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Büyük Kulüp</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>w235395223</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>amenity=social_club</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Büyük Kulüp (foursquare, Social Club, 1.0)</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="49" t="n"/>
+      <c r="I24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dalyan Club</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>w51814115</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>landuse=recreation_ground</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Dalyan Club (overture, social_or_community_service, 1.0)</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="49" t="n"/>
+      <c r="I25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Büyükada Rum Ortodoks Kabristanı</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>w132654555</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>amenity=grave_yard</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Büyükada Rum Ortodoks Kabristani (foursquare, Cemetery, 1.0)</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="49" t="n"/>
+      <c r="I26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Fenerbahçe Spor Kulübü Faruk Ilgaz Tesisleri</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>w235548988</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>landuse=recreation_ground</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Fenerbahçe SK Faruk Ilgaz Tesisleri (foursquare, Social Club, 0.89) | Fenerbahçe Spor Kulübü Konuk Evi - Faruk Ilgaz Tesisleri (foursquare, Housing Development, 0.9)</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="49" t="n"/>
+      <c r="I27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ada Beach Club</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>w595089732</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>leisure=beach_resort</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Ada Beach Club (overture, social_or_community_service, 1.0)</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="49" t="n"/>
+      <c r="I28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Rotapark Akademi</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>w1364587302</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>amenity=driving_school</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Rotapark Akademi (overture, specialty_school, 1.0)</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="49" t="n"/>
+      <c r="I29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>İizzet Baysal Huzurevi</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>w1539513173</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>amenity=social_facility</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>İzzet Baysal Huzurevi (overture, historic_site, 0.98)</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="49" t="n"/>
+      <c r="I30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Sakıp Sabancı Kandilli Eğitim ve Kültür Merkezi</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>r15258892</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Sakıp Sabancı Kandilli Egitim Ve Kultur Merkezi (overture, gym, 1.0)</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="49" t="n"/>
+      <c r="I31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Çubuklu Siloları</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>r0</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>historic=yes</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Çubuklu Silolar (overture, museum, 0.97)</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Müze → biletli kuralından. İBB'nin ücretsiz sergi/kültür mekânıysa açık-kamusal.</t>
+        </is>
+      </c>
+      <c r="H32" s="49" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-08 kararı</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Gaziosmanpaşa Belediyesi Yüzme Havuzu ve Spor Kompleksi</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>w818512567</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>leisure=fitness_centre</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Gaziosmanpaşa Belediyesi Yüzme Havuzu ve Spor Kompleksi (overture, gym, 1.0)</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="49" t="n"/>
+      <c r="I33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Pendik Balıkçı Barınağı</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>w812916672</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>leisure=marina</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Pendik Balıkcı Barınağı (overture, sport_or_recreation_club, 1.0)</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Marina: bir kısmı kamuya açık iskele / yürüyüş olabilir.</t>
+        </is>
+      </c>
+      <c r="H34" s="49" t="n"/>
+      <c r="I34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>ESBAŞ Katlı Otopark</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>w600269989</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>amenity=parking</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Esbaş Katlı Otopark (overture, parking, 1.0)</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="49" t="n"/>
+      <c r="I35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Kartal Kaymakamlığı</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>r13387169</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Kartal Kaymakamlığı (foursquare, Government Building, 1.0) | Kartal Kaymakamlığı (foursquare, City Hall, 1.0)</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="49" t="n"/>
+      <c r="I36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Kalamış Yelken Kulübü</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>w236166953</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>landuse=recreation_ground</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Kalamış Yelken Kulübü (foursquare, Harbor or Marina, 1.0)</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Kulüp; erişimsiz yerine davetli daha uygun olabilir.</t>
+        </is>
+      </c>
+      <c r="H37" s="49" t="n"/>
+      <c r="I37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Sancaktepe Metro İstasyonu</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>w1313330241</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Sancaktepe Metro İstasyonu (foursquare, Metro Station, 1.0)</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="49" t="n"/>
+      <c r="I38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul Büyükşehir Belediyesi Ek Hizmet Binası</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>w1052809788</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>İstanbul Büyükşehir Belediyesi Ek Hizmet Binası (foursquare, City Hall, 1.0)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="49" t="n"/>
+      <c r="I39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Red Go Kart</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>r0</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Red Go Kart (overture, sport_or_recreation_club, 1.0)</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="49" t="n"/>
+      <c r="I40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Artigiana Huzur Evi</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>w763290255</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>amenity=nursing_home</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Artigiana Huzur Evi (overture, civic_organization, 1.0)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="49" t="n"/>
+      <c r="I41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Yörükali Plajı</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>w526091858</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>leisure=beach_resort</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Yörük Ali Plajı (foursquare, Beach, 0.97)</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="49" t="n"/>
+      <c r="I42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Kilyos Kalesi</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>r13864528</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>historic=fort</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>erişimsiz</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Kilyos Kalesi (overture, military_site, 1.0) | Kilyos Kalesi (foursquare, Military Base, 1.0)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Askeri alan kaydından; kale ziyarete açıksa değişmeli.</t>
+        </is>
+      </c>
+      <c r="H43" s="49" t="n"/>
+      <c r="I43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Göktürk Botanik</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>w1148150945</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>landuse=greenhouse_horticulture</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Göktürk Botanik (overture, garden, 1.0)</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Özel bahçe / fidanlık olabilir.</t>
+        </is>
+      </c>
+      <c r="H44" s="49" t="n"/>
+      <c r="I44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>bambi garden</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>w940024286</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>landuse=allotments</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>biletli</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Bambi Garden (overture, event_venue, 1.0)</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="49" t="n"/>
+      <c r="I45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>VetAmerikan Hayvan Hastanesi</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>w1467139826</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>amenity=veterinary</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>açık-özel</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>VetAmerikan Hayvan Hastanesi (overture, animal_or_pet_service, 1.0)</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="49" t="n"/>
+      <c r="I46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Roma Bostanı</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>w246476621</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>landuse=yes</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Roma Bostanı (overture, historic_site, 1.0)</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="49" t="n"/>
+      <c r="I47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Gizli Bahçe</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>w572400902</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>landuse=greenhouse_horticulture</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Gizli Bahçe (foursquare, Botanical Garden, 1.0)</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="49" t="n"/>
+      <c r="I48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Pilavkaya</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>w938594157</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Pilav Kaya (foursquare, Beach, 0.95)</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="49" t="n"/>
+      <c r="I49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Elif Apartmanı</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>r0</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Elif apartmani (foursquare, Apartment or Condo, 1.0)</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr"/>
+      <c r="H50" s="49" t="n"/>
+      <c r="I50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Güzelce Su Kemeri</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>w1033475892</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>historic=aqueduct, man_made=bridge</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>açık-kamusal</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Güzelce Kemeri (overture, historic_site, 0.9)</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr"/>
+      <c r="H51" s="49" t="n"/>
+      <c r="I51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Beykoz GIS TM</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>w176290256</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>davetli</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Beykoz GIS TM (foursquare, Distribution Center, 1.0)</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr"/>
+      <c r="H52" s="49" t="n"/>
+      <c r="I52" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>